<commit_message>
Notas teste extra adicionadas
</commit_message>
<xml_diff>
--- a/Notas_EDO_IMPA_TECH.xlsx
+++ b/Notas_EDO_IMPA_TECH.xlsx
@@ -502,7 +502,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -552,6 +552,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -10077,8 +10081,8 @@
   <dimension ref="A1:B79"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.93"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15.02"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="44.93"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15.02"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10100,7 +10104,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>0.1</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10121,14 +10125,16 @@
       <c r="A6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="4"/>
+      <c r="B6" s="13" t="n">
+        <v>0.1</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
         <v>7</v>
       </c>
       <c r="B7" s="2" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10152,7 +10158,7 @@
         <v>10</v>
       </c>
       <c r="B10" s="2" t="n">
-        <v>0.05</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10168,7 +10174,7 @@
         <v>12</v>
       </c>
       <c r="B12" s="2" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10176,7 +10182,7 @@
         <v>13</v>
       </c>
       <c r="B13" s="2" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10190,7 +10196,7 @@
         <v>15</v>
       </c>
       <c r="B15" s="2" t="n">
-        <v>0.05</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10206,7 +10212,7 @@
         <v>17</v>
       </c>
       <c r="B17" s="2" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10214,7 +10220,7 @@
         <v>18</v>
       </c>
       <c r="B18" s="2" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10230,7 +10236,7 @@
         <v>20</v>
       </c>
       <c r="B20" s="2" t="n">
-        <v>0</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10238,7 +10244,7 @@
         <v>21</v>
       </c>
       <c r="B21" s="2" t="n">
-        <v>0</v>
+        <v>0.07</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10246,7 +10252,7 @@
         <v>22</v>
       </c>
       <c r="B22" s="2" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10254,7 +10260,7 @@
         <v>23</v>
       </c>
       <c r="B23" s="2" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10262,7 +10268,7 @@
         <v>24</v>
       </c>
       <c r="B24" s="2" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10284,7 +10290,7 @@
         <v>27</v>
       </c>
       <c r="B27" s="2" t="n">
-        <v>0.1</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10292,7 +10298,7 @@
         <v>28</v>
       </c>
       <c r="B28" s="2" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10308,7 +10314,7 @@
         <v>30</v>
       </c>
       <c r="B30" s="2" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10316,7 +10322,7 @@
         <v>31</v>
       </c>
       <c r="B31" s="2" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10332,7 +10338,7 @@
         <v>33</v>
       </c>
       <c r="B33" s="2" t="n">
-        <v>0.08</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10362,7 +10368,7 @@
         <v>37</v>
       </c>
       <c r="B37" s="2" t="n">
-        <v>0.05</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10378,7 +10384,7 @@
         <v>39</v>
       </c>
       <c r="B39" s="2" t="n">
-        <v>0</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10386,7 +10392,7 @@
         <v>40</v>
       </c>
       <c r="B40" s="2" t="n">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10394,7 +10400,7 @@
         <v>41</v>
       </c>
       <c r="B41" s="2" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10410,7 +10416,7 @@
         <v>43</v>
       </c>
       <c r="B43" s="2" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10418,7 +10424,7 @@
         <v>44</v>
       </c>
       <c r="B44" s="2" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10426,7 +10432,7 @@
         <v>45</v>
       </c>
       <c r="B45" s="2" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10466,7 +10472,7 @@
         <v>50</v>
       </c>
       <c r="B50" s="2" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10474,7 +10480,7 @@
         <v>51</v>
       </c>
       <c r="B51" s="2" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10482,7 +10488,7 @@
         <v>52</v>
       </c>
       <c r="B52" s="2" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10490,7 +10496,7 @@
         <v>53</v>
       </c>
       <c r="B53" s="2" t="n">
-        <v>0.03</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10498,7 +10504,7 @@
         <v>54</v>
       </c>
       <c r="B54" s="2" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10506,7 +10512,7 @@
         <v>55</v>
       </c>
       <c r="B55" s="2" t="n">
-        <v>0.1</v>
+        <v>0.07</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10514,7 +10520,7 @@
         <v>56</v>
       </c>
       <c r="B56" s="2" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10522,7 +10528,7 @@
         <v>57</v>
       </c>
       <c r="B57" s="2" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10570,7 +10576,7 @@
         <v>63</v>
       </c>
       <c r="B63" s="2" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10584,7 +10590,7 @@
         <v>65</v>
       </c>
       <c r="B65" s="2" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10592,7 +10598,7 @@
         <v>66</v>
       </c>
       <c r="B66" s="2" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10600,7 +10606,7 @@
         <v>67</v>
       </c>
       <c r="B67" s="2" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10630,7 +10636,7 @@
         <v>71</v>
       </c>
       <c r="B71" s="2" t="n">
-        <v>0.03</v>
+        <v>0</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10638,7 +10644,7 @@
         <v>72</v>
       </c>
       <c r="B72" s="2" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10646,7 +10652,7 @@
         <v>73</v>
       </c>
       <c r="B73" s="2" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10662,7 +10668,7 @@
         <v>75</v>
       </c>
       <c r="B75" s="2" t="n">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10670,7 +10676,7 @@
         <v>76</v>
       </c>
       <c r="B76" s="2" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10678,7 +10684,7 @@
         <v>77</v>
       </c>
       <c r="B77" s="2" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>